<commit_message>
feat(core): audit and harden scripts-core-install scope
- Translate .env.example, install.sh, setup_hermes.py, demo_tesorero.py,
  finance_sheet.py and all partenon-core/ files to English.
- Make install.sh and setup_hermes.py safe: no fake Hermes CLI URLs,
  graceful missing-CLI handling, clear next steps.
- Keep demo_tesorero.py runnable; rename outputs to sample_expenses.*.
- Add partenon-core/tools/config_loader.py and eval_loop.py stubs.
- Extend router.py to include partenon-brain profile.
- Harden workflow_engine.py and onboarding_engine.py against missing
  HBOS modules.
- Update MCP servers config and fix GBRAIN_DATABASE_URL env name.
</commit_message>
<xml_diff>
--- a/data/partenon-finance-template.xlsx
+++ b/data/partenon-finance-template.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ingresos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gastos Fijos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gastos Variables" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Proveedores" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,80 +443,80 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Indicador</t>
+          <t>Indicator</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ingresos mes actual</t>
+          <t>Current month income</t>
         </is>
       </c>
       <c r="B2" s="2">
-        <f>SUM(Ingresos[C])</f>
+        <f>SUM(Income!C:C)</f>
         <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Suma de hoja Ingresos</t>
+          <t>Sum of Income sheet</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Gastos fijos mes</t>
+          <t>Monthly fixed expenses</t>
         </is>
       </c>
       <c r="B3" s="2">
-        <f>SUMIF('Gastos Fijos'[C],"&lt;&gt;")</f>
+        <f>SUM('Fixed Expenses'!C:C)</f>
         <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Costos recurrentes</t>
+          <t>Recurring costs</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Gastos variables mes</t>
+          <t>Monthly variable expenses</t>
         </is>
       </c>
       <c r="B4" s="2">
-        <f>SUMIF('Gastos Variables'[C],"&lt;&gt;")</f>
+        <f>SUM('Variable Expenses'!C:C)</f>
         <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Costos proporcionales</t>
+          <t>Proportional costs</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Margen estimado</t>
+          <t>Estimated margin</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -525,18 +525,18 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Ingresos - gastos</t>
+          <t>Income - expenses</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Proveedores activos</t>
+          <t>Active suppliers</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTA(Proveedores[A])-1</f>
+        <f>COUNTA(Suppliers!A:A)-1</f>
         <v/>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -555,37 +555,37 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Monto</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Canal</t>
+          <t>Channel</t>
         </is>
       </c>
     </row>
@@ -603,37 +603,37 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Monto</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Frecuencia</t>
+          <t>Frequency</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Proveedor</t>
+          <t>Supplier</t>
         </is>
       </c>
     </row>
@@ -651,37 +651,37 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Monto</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Categoria</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Proveedor</t>
+          <t>Supplier</t>
         </is>
       </c>
     </row>
@@ -699,37 +699,37 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Contacto</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Pago habitual</t>
+          <t>Usual payment</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Calificacion</t>
+          <t>Rating</t>
         </is>
       </c>
     </row>

</xml_diff>